<commit_message>
Reset Excel Table for ARGON-02
</commit_message>
<xml_diff>
--- a/FM-MN-07_ARGON-02.xlsx
+++ b/FM-MN-07_ARGON-02.xlsx
@@ -1768,11 +1768,7 @@
           <t>ตรวจสภาพความพรัอมโดยรวมของเครื่อง</t>
         </is>
       </c>
-      <c r="C6" s="26" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C6" s="26" t="inlineStr"/>
       <c r="D6" s="26" t="inlineStr"/>
       <c r="E6" s="26" t="inlineStr"/>
       <c r="F6" s="26" t="inlineStr"/>
@@ -1813,11 +1809,7 @@
           <t xml:space="preserve">เช็ค  BREAKER  เพื่อเช็คระบบไฟฟ้า ตามตำแหน่งไฟ โชว์  และ SWITCH  ต่าง ๆ </t>
         </is>
       </c>
-      <c r="C7" s="26" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C7" s="26" t="inlineStr"/>
       <c r="D7" s="26" t="inlineStr"/>
       <c r="E7" s="26" t="inlineStr"/>
       <c r="F7" s="26" t="inlineStr"/>
@@ -1899,11 +1891,7 @@
           <t>ตรวจุดต่อของสายก๊าช  ARGON  ก่อนว่ารั่วหรือไม่</t>
         </is>
       </c>
-      <c r="C9" s="26" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C9" s="26" t="inlineStr"/>
       <c r="D9" s="26" t="inlineStr"/>
       <c r="E9" s="26" t="inlineStr"/>
       <c r="F9" s="26" t="inlineStr"/>
@@ -2102,11 +2090,7 @@
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="7" t="n"/>
       <c r="B14" s="6" t="n"/>
-      <c r="C14" s="42" t="inlineStr">
-        <is>
-          <t>อินทัช เป็นสุข</t>
-        </is>
-      </c>
+      <c r="C14" s="42" t="inlineStr"/>
       <c r="D14" s="40" t="inlineStr"/>
       <c r="E14" s="40" t="inlineStr"/>
       <c r="F14" s="40" t="inlineStr"/>

</xml_diff>

<commit_message>
Direct Write Excel for ARGON-02 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_ARGON-02.xlsx
+++ b/FM-MN-07_ARGON-02.xlsx
@@ -1773,7 +1773,11 @@
       <c r="E6" s="26" t="inlineStr"/>
       <c r="F6" s="26" t="inlineStr"/>
       <c r="G6" s="26" t="inlineStr"/>
-      <c r="H6" s="26" t="inlineStr"/>
+      <c r="H6" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="26" t="inlineStr"/>
       <c r="J6" s="26" t="inlineStr"/>
       <c r="K6" s="26" t="inlineStr"/>
@@ -1814,7 +1818,11 @@
       <c r="E7" s="26" t="inlineStr"/>
       <c r="F7" s="26" t="inlineStr"/>
       <c r="G7" s="26" t="inlineStr"/>
-      <c r="H7" s="26" t="inlineStr"/>
+      <c r="H7" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="26" t="inlineStr"/>
       <c r="J7" s="26" t="inlineStr"/>
       <c r="K7" s="26" t="inlineStr"/>
@@ -1855,7 +1863,11 @@
       <c r="E8" s="26" t="inlineStr"/>
       <c r="F8" s="26" t="inlineStr"/>
       <c r="G8" s="26" t="inlineStr"/>
-      <c r="H8" s="26" t="inlineStr"/>
+      <c r="H8" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="26" t="inlineStr"/>
       <c r="J8" s="26" t="inlineStr"/>
       <c r="K8" s="26" t="inlineStr"/>
@@ -1896,7 +1908,11 @@
       <c r="E9" s="26" t="inlineStr"/>
       <c r="F9" s="26" t="inlineStr"/>
       <c r="G9" s="26" t="inlineStr"/>
-      <c r="H9" s="26" t="inlineStr"/>
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="26" t="inlineStr"/>
       <c r="J9" s="26" t="inlineStr"/>
       <c r="K9" s="26" t="inlineStr"/>
@@ -1937,7 +1953,11 @@
       <c r="E10" s="26" t="inlineStr"/>
       <c r="F10" s="26" t="inlineStr"/>
       <c r="G10" s="26" t="inlineStr"/>
-      <c r="H10" s="26" t="inlineStr"/>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="26" t="inlineStr"/>
       <c r="J10" s="26" t="inlineStr"/>
       <c r="K10" s="26" t="inlineStr"/>
@@ -1978,7 +1998,11 @@
       <c r="E11" s="26" t="inlineStr"/>
       <c r="F11" s="26" t="inlineStr"/>
       <c r="G11" s="26" t="inlineStr"/>
-      <c r="H11" s="26" t="inlineStr"/>
+      <c r="H11" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I11" s="26" t="inlineStr"/>
       <c r="J11" s="26" t="inlineStr"/>
       <c r="K11" s="26" t="inlineStr"/>
@@ -2019,7 +2043,11 @@
       <c r="E12" s="26" t="inlineStr"/>
       <c r="F12" s="26" t="inlineStr"/>
       <c r="G12" s="26" t="inlineStr"/>
-      <c r="H12" s="26" t="inlineStr"/>
+      <c r="H12" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I12" s="26" t="inlineStr"/>
       <c r="J12" s="26" t="inlineStr"/>
       <c r="K12" s="26" t="inlineStr"/>
@@ -2060,7 +2088,11 @@
       <c r="E13" s="26" t="inlineStr"/>
       <c r="F13" s="26" t="inlineStr"/>
       <c r="G13" s="26" t="inlineStr"/>
-      <c r="H13" s="26" t="inlineStr"/>
+      <c r="H13" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I13" s="26" t="inlineStr"/>
       <c r="J13" s="26" t="inlineStr"/>
       <c r="K13" s="26" t="inlineStr"/>
@@ -2095,7 +2127,11 @@
       <c r="E14" s="40" t="inlineStr"/>
       <c r="F14" s="40" t="inlineStr"/>
       <c r="G14" s="40" t="inlineStr"/>
-      <c r="H14" s="40" t="inlineStr"/>
+      <c r="H14" s="42" t="inlineStr">
+        <is>
+          <t>อินทัช เป็นสุข</t>
+        </is>
+      </c>
       <c r="I14" s="40" t="inlineStr"/>
       <c r="J14" s="40" t="inlineStr"/>
       <c r="K14" s="40" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for ARGON-02 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_ARGON-02.xlsx
+++ b/FM-MN-07_ARGON-02.xlsx
@@ -1778,7 +1778,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="26" t="inlineStr"/>
+      <c r="I6" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="26" t="inlineStr"/>
       <c r="K6" s="26" t="inlineStr"/>
       <c r="L6" s="26" t="inlineStr"/>
@@ -1823,7 +1827,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="26" t="inlineStr"/>
+      <c r="I7" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="26" t="inlineStr"/>
       <c r="K7" s="26" t="inlineStr"/>
       <c r="L7" s="26" t="inlineStr"/>
@@ -1868,7 +1876,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="26" t="inlineStr"/>
+      <c r="I8" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="26" t="inlineStr"/>
       <c r="K8" s="26" t="inlineStr"/>
       <c r="L8" s="26" t="inlineStr"/>
@@ -1913,7 +1925,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="26" t="inlineStr"/>
+      <c r="I9" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="26" t="inlineStr"/>
       <c r="K9" s="26" t="inlineStr"/>
       <c r="L9" s="26" t="inlineStr"/>
@@ -1958,7 +1974,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="26" t="inlineStr"/>
+      <c r="I10" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="26" t="inlineStr"/>
       <c r="K10" s="26" t="inlineStr"/>
       <c r="L10" s="26" t="inlineStr"/>
@@ -2003,7 +2023,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I11" s="26" t="inlineStr"/>
+      <c r="I11" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J11" s="26" t="inlineStr"/>
       <c r="K11" s="26" t="inlineStr"/>
       <c r="L11" s="26" t="inlineStr"/>
@@ -2048,7 +2072,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I12" s="26" t="inlineStr"/>
+      <c r="I12" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J12" s="26" t="inlineStr"/>
       <c r="K12" s="26" t="inlineStr"/>
       <c r="L12" s="26" t="inlineStr"/>
@@ -2093,7 +2121,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I13" s="26" t="inlineStr"/>
+      <c r="I13" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J13" s="26" t="inlineStr"/>
       <c r="K13" s="26" t="inlineStr"/>
       <c r="L13" s="26" t="inlineStr"/>
@@ -2132,7 +2164,11 @@
           <t>อินทัช เป็นสุข</t>
         </is>
       </c>
-      <c r="I14" s="40" t="inlineStr"/>
+      <c r="I14" s="42" t="inlineStr">
+        <is>
+          <t>อินทัช เป็นสุข</t>
+        </is>
+      </c>
       <c r="J14" s="40" t="inlineStr"/>
       <c r="K14" s="40" t="inlineStr"/>
       <c r="L14" s="40" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for ARGON-02 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_ARGON-02.xlsx
+++ b/FM-MN-07_ARGON-02.xlsx
@@ -1785,7 +1785,11 @@
       </c>
       <c r="J6" s="26" t="inlineStr"/>
       <c r="K6" s="26" t="inlineStr"/>
-      <c r="L6" s="26" t="inlineStr"/>
+      <c r="L6" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="26" t="inlineStr"/>
       <c r="N6" s="26" t="inlineStr"/>
       <c r="O6" s="26" t="inlineStr"/>
@@ -1834,7 +1838,11 @@
       </c>
       <c r="J7" s="26" t="inlineStr"/>
       <c r="K7" s="26" t="inlineStr"/>
-      <c r="L7" s="26" t="inlineStr"/>
+      <c r="L7" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="26" t="inlineStr"/>
       <c r="N7" s="26" t="inlineStr"/>
       <c r="O7" s="26" t="inlineStr"/>
@@ -1883,7 +1891,11 @@
       </c>
       <c r="J8" s="26" t="inlineStr"/>
       <c r="K8" s="26" t="inlineStr"/>
-      <c r="L8" s="26" t="inlineStr"/>
+      <c r="L8" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="26" t="inlineStr"/>
       <c r="N8" s="26" t="inlineStr"/>
       <c r="O8" s="26" t="inlineStr"/>
@@ -1932,7 +1944,11 @@
       </c>
       <c r="J9" s="26" t="inlineStr"/>
       <c r="K9" s="26" t="inlineStr"/>
-      <c r="L9" s="26" t="inlineStr"/>
+      <c r="L9" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="26" t="inlineStr"/>
       <c r="N9" s="26" t="inlineStr"/>
       <c r="O9" s="26" t="inlineStr"/>
@@ -1981,7 +1997,11 @@
       </c>
       <c r="J10" s="26" t="inlineStr"/>
       <c r="K10" s="26" t="inlineStr"/>
-      <c r="L10" s="26" t="inlineStr"/>
+      <c r="L10" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="26" t="inlineStr"/>
       <c r="N10" s="26" t="inlineStr"/>
       <c r="O10" s="26" t="inlineStr"/>
@@ -2030,7 +2050,11 @@
       </c>
       <c r="J11" s="26" t="inlineStr"/>
       <c r="K11" s="26" t="inlineStr"/>
-      <c r="L11" s="26" t="inlineStr"/>
+      <c r="L11" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M11" s="26" t="inlineStr"/>
       <c r="N11" s="26" t="inlineStr"/>
       <c r="O11" s="26" t="inlineStr"/>
@@ -2079,7 +2103,11 @@
       </c>
       <c r="J12" s="26" t="inlineStr"/>
       <c r="K12" s="26" t="inlineStr"/>
-      <c r="L12" s="26" t="inlineStr"/>
+      <c r="L12" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M12" s="26" t="inlineStr"/>
       <c r="N12" s="26" t="inlineStr"/>
       <c r="O12" s="26" t="inlineStr"/>
@@ -2128,7 +2156,11 @@
       </c>
       <c r="J13" s="26" t="inlineStr"/>
       <c r="K13" s="26" t="inlineStr"/>
-      <c r="L13" s="26" t="inlineStr"/>
+      <c r="L13" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M13" s="26" t="inlineStr"/>
       <c r="N13" s="26" t="inlineStr"/>
       <c r="O13" s="26" t="inlineStr"/>
@@ -2171,7 +2203,11 @@
       </c>
       <c r="J14" s="40" t="inlineStr"/>
       <c r="K14" s="40" t="inlineStr"/>
-      <c r="L14" s="40" t="inlineStr"/>
+      <c r="L14" s="42" t="inlineStr">
+        <is>
+          <t>อนุสรณ์  ชื่นแฉ่ง</t>
+        </is>
+      </c>
       <c r="M14" s="40" t="inlineStr"/>
       <c r="N14" s="40" t="inlineStr"/>
       <c r="O14" s="40" t="inlineStr"/>

</xml_diff>